<commit_message>
se obtiene popularidad directo del endpoint de los artistas, quitando el calculo de popularidad por promedio del top 10 tracks
</commit_message>
<xml_diff>
--- a/artists.xlsx
+++ b/artists.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspaces\Spotipy-Playlists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCCABC7-C5FA-4B93-815C-98AB0D894611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F5DCCEA-6220-4514-B445-3CD822C41BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
   <si>
     <t>artist_id</t>
   </si>
@@ -65,9 +65,6 @@
     <t>La Dosis</t>
   </si>
   <si>
-    <t>Mariano Bermudez</t>
-  </si>
-  <si>
     <t>La Bocha 12</t>
   </si>
   <si>
@@ -119,9 +116,6 @@
     <t>1i09cLSfZNYlP8yx7XbK6M</t>
   </si>
   <si>
-    <t>Agata Uruguay</t>
-  </si>
-  <si>
     <t>2lT39ZyCy8SWSrTWvWlksN</t>
   </si>
   <si>
@@ -161,9 +155,6 @@
     <t>10A9ktGErbFGnyn1VplHND</t>
   </si>
   <si>
-    <t>Bocha Lozano y La Vieja Escuela</t>
-  </si>
-  <si>
     <t>3wzyB2hhQSrqUE4crKX64Y</t>
   </si>
   <si>
@@ -179,9 +170,6 @@
     <t>3F4XOLVuGkMDSIGu2Kn33M</t>
   </si>
   <si>
-    <t>Carlos Corti y Los Muchachos</t>
-  </si>
-  <si>
     <t>76V41O7m8rFTOJllXHBo9G</t>
   </si>
   <si>
@@ -200,24 +188,9 @@
     <t>Como Keda</t>
   </si>
   <si>
-    <t>6mMF00MGSqk8MT3c31YRSg</t>
-  </si>
-  <si>
-    <t>Como Suena</t>
-  </si>
-  <si>
     <t>5pjGkQyoECqaaQLMn9z6he</t>
   </si>
   <si>
-    <t>Damián Lescano</t>
-  </si>
-  <si>
-    <t>6oWte5YNjECFloePYCVkle</t>
-  </si>
-  <si>
-    <t>Daniel Tata Torres</t>
-  </si>
-  <si>
     <t>4AFl787KWUdOe2Ufjd3IqK</t>
   </si>
   <si>
@@ -227,15 +200,9 @@
     <t>1ZFsNDKnDi567xFAvS6vHH</t>
   </si>
   <si>
-    <t>Diego El Cantante</t>
-  </si>
-  <si>
     <t>1IYPsxunWpJvDYA1Por8dI</t>
   </si>
   <si>
-    <t>Diego Ríos</t>
-  </si>
-  <si>
     <t>1fN7fYrsFplBYEOOVxvAvK</t>
   </si>
   <si>
@@ -245,39 +212,15 @@
     <t>0annXurxTVJKs4QqOqdwGR</t>
   </si>
   <si>
-    <t>El Gucci y su Banda</t>
-  </si>
-  <si>
     <t>0stzICt2pSbffNTrQekkPT</t>
   </si>
   <si>
-    <t>El Karnal y Su Banda</t>
-  </si>
-  <si>
-    <t>7tQNgiLNw9eeWJqJ5bCApk</t>
-  </si>
-  <si>
-    <t>El León de la Plena</t>
-  </si>
-  <si>
-    <t>1LSYfRidvKN3sUXOg8HDWC</t>
-  </si>
-  <si>
-    <t>El Mala</t>
-  </si>
-  <si>
     <t>1jEmkSA4MX2EjZE9J2dAR9</t>
   </si>
   <si>
     <t>El Plan</t>
   </si>
   <si>
-    <t>7HSeegdmjLYRJpkOYIaZIW</t>
-  </si>
-  <si>
-    <t>El Reja</t>
-  </si>
-  <si>
     <t>4nTNHKAVWQyqnvRuBW4N4V</t>
   </si>
   <si>
@@ -308,12 +251,6 @@
     <t>Fede Rojas</t>
   </si>
   <si>
-    <t>3CoHirtwCpNmEHyoxJoBtg</t>
-  </si>
-  <si>
-    <t>Fer Costa</t>
-  </si>
-  <si>
     <t>5HUPhcBE9Bg1LLnFrhRcOy</t>
   </si>
   <si>
@@ -347,9 +284,6 @@
     <t>30YXApUmvoMSvQ41AuUUNv</t>
   </si>
   <si>
-    <t>Javier Leite</t>
-  </si>
-  <si>
     <t>48k3R82F45Jaa4C8GDnLOu</t>
   </si>
   <si>
@@ -374,12 +308,6 @@
     <t>Katy Bordagorria</t>
   </si>
   <si>
-    <t>4wld5HDVMVy9I6MnPqjzFH</t>
-  </si>
-  <si>
-    <t>Ke Kumbia</t>
-  </si>
-  <si>
     <t>7qyphxox1qgcpTUHbVP5PK</t>
   </si>
   <si>
@@ -410,18 +338,6 @@
     <t>La Dupla</t>
   </si>
   <si>
-    <t>0YNTZqoGsHjDMFUPbm2jGJ</t>
-  </si>
-  <si>
-    <t>La Furia</t>
-  </si>
-  <si>
-    <t>5b0t98sO8PmHcr3eAXcSMg</t>
-  </si>
-  <si>
-    <t>La Fase-Buk</t>
-  </si>
-  <si>
     <t>2JJXJsbTyotc9Rm0KWSTdQ</t>
   </si>
   <si>
@@ -431,27 +347,9 @@
     <t>5zsJoBmoHM1A6jEoEcNmMv</t>
   </si>
   <si>
-    <t>La NT y Los Siniestros</t>
-  </si>
-  <si>
     <t>07y4PkqTJCaJAjQ1jCKoJx</t>
   </si>
   <si>
-    <t>La Penúltima</t>
-  </si>
-  <si>
-    <t>4oZolC0sCwCAKqsNXfRlVS</t>
-  </si>
-  <si>
-    <t>The la Planta</t>
-  </si>
-  <si>
-    <t>75HTvu7Rywwrm4K2yR6xie</t>
-  </si>
-  <si>
-    <t>La Revancha</t>
-  </si>
-  <si>
     <t>2dlmYYzcmde3ej5FpNtg7y</t>
   </si>
   <si>
@@ -494,24 +392,12 @@
     <t>Letan</t>
   </si>
   <si>
-    <t>1kyy6AW7C6Rr2jrYwz95Gi</t>
-  </si>
-  <si>
-    <t>Lira</t>
-  </si>
-  <si>
     <t>5v2YVowYeNRB1vK1JTBSP0</t>
   </si>
   <si>
     <t>Los Bembones</t>
   </si>
   <si>
-    <t>5mLvRBeI5T7w08iWtK7FXu</t>
-  </si>
-  <si>
-    <t>Los Fatales</t>
-  </si>
-  <si>
     <t>6WrhdoSkwNxeTzjtdLfnPU</t>
   </si>
   <si>
@@ -524,30 +410,12 @@
     <t>Los Pikantes</t>
   </si>
   <si>
-    <t>4oLMD76t4pIw2dXsF4VlrI</t>
-  </si>
-  <si>
-    <t>Los Torres</t>
-  </si>
-  <si>
     <t>5nsESBMEZ2TwECdxPPgmbB</t>
   </si>
   <si>
     <t>Luaa</t>
   </si>
   <si>
-    <t>1AIGPpwjs3zZXT7cJIYEOM</t>
-  </si>
-  <si>
-    <t>Lucas Bunker</t>
-  </si>
-  <si>
-    <t>24QqF0upv6pRO6fMI4jIuL</t>
-  </si>
-  <si>
-    <t>Lucas Corbo</t>
-  </si>
-  <si>
     <t>0WnP62TjkFfRrt52yE8zcX</t>
   </si>
   <si>
@@ -560,18 +428,6 @@
     <t>Luciana</t>
   </si>
   <si>
-    <t>2gHzzL0wGI0XXNuOzcbUe8</t>
-  </si>
-  <si>
-    <t>Lucrecia</t>
-  </si>
-  <si>
-    <t>1SDdOa5e5D3XIR2t8Mb3dm</t>
-  </si>
-  <si>
-    <t>L'Autentika</t>
-  </si>
-  <si>
     <t>13PNcLm9aol5SG4hPn1UUi</t>
   </si>
   <si>
@@ -581,9 +437,6 @@
     <t>2dSeDxBzKslmct6a2R4JYZ</t>
   </si>
   <si>
-    <t>Majo y al del 13</t>
-  </si>
-  <si>
     <t>2weGfox1CWg9HmmwDgcjey</t>
   </si>
   <si>
@@ -602,12 +455,6 @@
     <t>Mariela Barboza</t>
   </si>
   <si>
-    <t>4SgKWjM7cJDCh2aY9H4HZf</t>
-  </si>
-  <si>
-    <t>Marka Akme</t>
-  </si>
-  <si>
     <t>1TndreWtLjfAlywnkm966g</t>
   </si>
   <si>
@@ -653,21 +500,9 @@
     <t>6SGCqG5HEr5gFZR9ct8wID</t>
   </si>
   <si>
-    <t>Matías Valdez</t>
-  </si>
-  <si>
-    <t>7HW35ytaUKrvvpGoL9wYOz</t>
-  </si>
-  <si>
-    <t>Max Fernández</t>
-  </si>
-  <si>
     <t>2UnGWnrqDZPjWNVRWj5Mae</t>
   </si>
   <si>
-    <t>Maxi Álvarez</t>
-  </si>
-  <si>
     <t>2qVxbJYW5xbslFjhPBGjXY</t>
   </si>
   <si>
@@ -686,36 +521,12 @@
     <t>Natanael Segovia</t>
   </si>
   <si>
-    <t>3ihnywVzkqr6nZ7sb9Z4tr</t>
-  </si>
-  <si>
-    <t>Nati Ferrero</t>
-  </si>
-  <si>
     <t>1OicNKNw1iMMSpFm2VIJwv</t>
   </si>
   <si>
-    <t>Nico Conca y Su Banda</t>
-  </si>
-  <si>
     <t>51YgtNDifRmwn2hPhAVHCi</t>
   </si>
   <si>
-    <t>Nicolás Castillo</t>
-  </si>
-  <si>
-    <t>1cMayct0l7y4gE5qFSSCm9</t>
-  </si>
-  <si>
-    <t>Numi Martínez</t>
-  </si>
-  <si>
-    <t>6L2DyVdMndLfvkAelI8vFe</t>
-  </si>
-  <si>
-    <t>ONE PLAY</t>
-  </si>
-  <si>
     <t>6hdAcFnlOI70rcco0TXaH6</t>
   </si>
   <si>
@@ -734,12 +545,6 @@
     <t>Paulino</t>
   </si>
   <si>
-    <t>1l6UgL5G16tId4qoYH8qJn</t>
-  </si>
-  <si>
-    <t>Pushi</t>
-  </si>
-  <si>
     <t>5sXtJMLiU5jgZzrPmaj6Gv</t>
   </si>
   <si>
@@ -758,18 +563,12 @@
     <t>Santino</t>
   </si>
   <si>
-    <t>2TjBEdasWbKTGJnfj5a1ea</t>
-  </si>
-  <si>
     <t>Seba Torres</t>
   </si>
   <si>
     <t>5yUamcZHhXrqRxR768n4YT</t>
   </si>
   <si>
-    <t>Seba Pereyra</t>
-  </si>
-  <si>
     <t>4qywsc4qd533a1CWJUtOR3</t>
   </si>
   <si>
@@ -794,12 +593,6 @@
     <t>Sonido Cristal</t>
   </si>
   <si>
-    <t>1BfR4gQyjlhLAssULX0wDr</t>
-  </si>
-  <si>
-    <t>Valeria Gau</t>
-  </si>
-  <si>
     <t>04vVNmaKhinxxW4eCJIyX7</t>
   </si>
   <si>
@@ -818,96 +611,21 @@
     <t>Vanesa Britos</t>
   </si>
   <si>
-    <t>44hJXrVhoyA1fV1dn4wdHC</t>
-  </si>
-  <si>
-    <t>VI-EM</t>
-  </si>
-  <si>
     <t>2ErBBWTmb2KkwXVDUaPeBP</t>
   </si>
   <si>
-    <t>Yesty Prieto</t>
-  </si>
-  <si>
-    <t>2qmA5QmaGZH3ky4qq25d1m</t>
-  </si>
-  <si>
-    <t>Agus Padilla</t>
-  </si>
-  <si>
-    <t>2WhGojaMjv4VVn2HQSqrLM</t>
-  </si>
-  <si>
-    <t>Agustín Casanova</t>
-  </si>
-  <si>
-    <t>474st1ZFIh7IOiUcw9ojHd</t>
-  </si>
-  <si>
-    <t>AX-13</t>
-  </si>
-  <si>
-    <t>4e3lv5qRgFpdILdEOHchbn</t>
-  </si>
-  <si>
-    <t>Chocolate</t>
-  </si>
-  <si>
-    <t>0J65S0gB0D1gDEd0hK196k</t>
-  </si>
-  <si>
-    <t>Dame 5</t>
-  </si>
-  <si>
-    <t>2LI6qhH2fF1uoJpmquvoCn</t>
-  </si>
-  <si>
-    <t>Dessia El Otro</t>
-  </si>
-  <si>
     <t>77xPFPxusAy6VVAXc6pWFg</t>
   </si>
   <si>
     <t>Gonzalo Castillo</t>
   </si>
   <si>
-    <t>1I7vbkqIHVffUHHmmXWAYr</t>
-  </si>
-  <si>
-    <t>JULIETTA</t>
-  </si>
-  <si>
-    <t>5KQX0Ui06LVm6PApyicRFK</t>
-  </si>
-  <si>
-    <t>Rombai</t>
-  </si>
-  <si>
-    <t>5nAsuOI0lqqbii7YFCh7cB</t>
-  </si>
-  <si>
-    <t>Fer Vazquez</t>
-  </si>
-  <si>
-    <t>39x7olLItlZSz0uodtTEeG</t>
-  </si>
-  <si>
-    <t>Sole Ramírez</t>
-  </si>
-  <si>
     <t>3bSypudQFjg4tNIKgoH83Z</t>
   </si>
   <si>
     <t>Sonido Profesional</t>
   </si>
   <si>
-    <t>29W4Fw8TDGfXD7C9EjJkzc</t>
-  </si>
-  <si>
-    <t>Sonido de la Costa</t>
-  </si>
-  <si>
     <t>0R7hVTyBZQ9ApxMtDEAwyL</t>
   </si>
   <si>
@@ -920,34 +638,76 @@
     <t>Soy tu Sol</t>
   </si>
   <si>
-    <t>2gg8RhbAVd4tW7LdZZ5RvR</t>
-  </si>
-  <si>
-    <t>Thian the Producer</t>
-  </si>
-  <si>
-    <t>28hVuLtRLgq1HSXM8jI7gA</t>
-  </si>
-  <si>
-    <t>UNA+</t>
-  </si>
-  <si>
-    <t>7zREGj8GMl9UrDa6NPLi0H</t>
-  </si>
-  <si>
-    <t>Meri Deal</t>
-  </si>
-  <si>
-    <t>4cV73y9UlkKTCIWbuP2hbG</t>
-  </si>
-  <si>
-    <t>Bauti Mascia</t>
-  </si>
-  <si>
-    <t>4GepMkTgrIZECoCC55vqjW</t>
-  </si>
-  <si>
-    <t>Marama</t>
+    <t>Agata</t>
+  </si>
+  <si>
+    <t>Bocha Lozano</t>
+  </si>
+  <si>
+    <t>Carlos Corti</t>
+  </si>
+  <si>
+    <t>Damian Lescano</t>
+  </si>
+  <si>
+    <t>Diego el Cantante</t>
+  </si>
+  <si>
+    <t>Diego Rios</t>
+  </si>
+  <si>
+    <t>El Gucci</t>
+  </si>
+  <si>
+    <t>El Karnal</t>
+  </si>
+  <si>
+    <t>Javier Leite 1</t>
+  </si>
+  <si>
+    <t>La NT &amp; Los Siniestros</t>
+  </si>
+  <si>
+    <t>La Penultima</t>
+  </si>
+  <si>
+    <t>Majo y la del 13</t>
+  </si>
+  <si>
+    <t>Mariano Bermúdez</t>
+  </si>
+  <si>
+    <t>Matias Valdez</t>
+  </si>
+  <si>
+    <t>Maxi Alvarez</t>
+  </si>
+  <si>
+    <t>Nico Conca</t>
+  </si>
+  <si>
+    <t>Nicolas Castillo</t>
+  </si>
+  <si>
+    <t>3GxnN9pvXJyp0s5zeBKqYQ</t>
+  </si>
+  <si>
+    <t>El Desakato</t>
+  </si>
+  <si>
+    <t>0nDC68Q70JH7P5Fs5KyVxq</t>
+  </si>
+  <si>
+    <t>Santiago Pintos</t>
+  </si>
+  <si>
+    <t>6029g3SIplZfI0tk5LM7Rr</t>
+  </si>
+  <si>
+    <t>Tamo Activo</t>
+  </si>
+  <si>
+    <t>Yesti Prieto</t>
   </si>
 </sst>
 </file>
@@ -1014,10 +774,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B8818374-0E59-463B-B82D-4169E37A15D7}" name="Tabla2" displayName="Tabla2" ref="A1:B152" totalsRowShown="0">
-  <autoFilter ref="A1:B152" xr:uid="{B8818374-0E59-463B-B82D-4169E37A15D7}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B149">
-    <sortCondition ref="B1:B149"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B8818374-0E59-463B-B82D-4169E37A15D7}" name="Tabla2" displayName="Tabla2" ref="A1:B112" totalsRowShown="0">
+  <autoFilter ref="A1:B112" xr:uid="{B8818374-0E59-463B-B82D-4169E37A15D7}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B2">
+    <sortCondition ref="B1:B2"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0B640077-FDFE-4CE3-8070-C3013D7400F3}" name="artist_id"/>
@@ -1290,7 +1050,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B152"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
@@ -1307,26 +1067,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>264</v>
+        <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>265</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>266</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>267</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1371,90 +1131,90 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>268</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>269</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B12" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>41</v>
+        <v>202</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="B18" t="s">
-        <v>51</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>270</v>
+        <v>51</v>
       </c>
       <c r="B19" t="s">
-        <v>271</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B20" t="s">
-        <v>53</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -1462,23 +1222,23 @@
         <v>54</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>272</v>
+        <v>55</v>
       </c>
       <c r="B22" t="s">
-        <v>273</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -1486,119 +1246,119 @@
         <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>207</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>13</v>
+        <v>59</v>
       </c>
       <c r="B25" t="s">
-        <v>3</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>274</v>
+        <v>61</v>
       </c>
       <c r="B26" t="s">
-        <v>275</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" t="s">
         <v>64</v>
-      </c>
-      <c r="B29" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>192</v>
       </c>
       <c r="B37" t="s">
-        <v>81</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>17</v>
+        <v>81</v>
       </c>
       <c r="B38" t="s">
-        <v>7</v>
+        <v>208</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -1627,194 +1387,194 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="B42" t="s">
-        <v>89</v>
+        <v>5</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B43" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B44" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>282</v>
+        <v>19</v>
       </c>
       <c r="B45" t="s">
-        <v>283</v>
+        <v>9</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>276</v>
+        <v>17</v>
       </c>
       <c r="B50" t="s">
-        <v>277</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B51" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B52" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B53" t="s">
-        <v>107</v>
+        <v>209</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>108</v>
+        <v>15</v>
       </c>
       <c r="B54" t="s">
-        <v>109</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>15</v>
+        <v>103</v>
       </c>
       <c r="B55" t="s">
-        <v>5</v>
+        <v>210</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>278</v>
+        <v>104</v>
       </c>
       <c r="B56" t="s">
-        <v>279</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>110</v>
+        <v>21</v>
       </c>
       <c r="B57" t="s">
-        <v>111</v>
+        <v>11</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B59" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="B60" t="s">
-        <v>10</v>
+        <v>111</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B61" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B62" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B63" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>21</v>
+        <v>118</v>
       </c>
       <c r="B64" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>18</v>
+        <v>120</v>
       </c>
       <c r="B65" t="s">
-        <v>8</v>
+        <v>121</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -1827,42 +1587,42 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B67" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>124</v>
+        <v>13</v>
       </c>
       <c r="B68" t="s">
-        <v>125</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B69" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B70" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>16</v>
+        <v>130</v>
       </c>
       <c r="B71" t="s">
-        <v>6</v>
+        <v>131</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -1870,263 +1630,263 @@
         <v>132</v>
       </c>
       <c r="B72" t="s">
-        <v>133</v>
+        <v>211</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B73" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B74" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B75" t="s">
-        <v>12</v>
+        <v>212</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B76" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B77" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B78" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B80" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>176</v>
+        <v>147</v>
       </c>
       <c r="B81" t="s">
-        <v>177</v>
+        <v>148</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" t="s">
         <v>150</v>
-      </c>
-      <c r="B82" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>151</v>
+      </c>
+      <c r="B83" t="s">
         <v>152</v>
-      </c>
-      <c r="B83" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B84" t="s">
-        <v>155</v>
+        <v>213</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B85" t="s">
-        <v>157</v>
+        <v>214</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B86" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B87" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B88" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B89" t="s">
-        <v>165</v>
+        <v>215</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="B90" t="s">
-        <v>4</v>
+        <v>216</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B91" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B92" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>170</v>
+        <v>217</v>
       </c>
       <c r="B93" t="s">
-        <v>171</v>
+        <v>218</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>172</v>
+        <v>22</v>
       </c>
       <c r="B94" t="s">
-        <v>173</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="B95" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="B96" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="B97" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>182</v>
+        <v>219</v>
       </c>
       <c r="B98" t="s">
-        <v>183</v>
+        <v>220</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="B99" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>19</v>
+        <v>176</v>
       </c>
       <c r="B100" t="s">
-        <v>9</v>
+        <v>175</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="B101" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="B102" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="B103" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="B104" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
@@ -2155,362 +1915,42 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
       <c r="B108" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="B109" t="s">
-        <v>203</v>
+        <v>187</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="B110" t="s">
-        <v>205</v>
+        <v>186</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>206</v>
+        <v>189</v>
       </c>
       <c r="B111" t="s">
-        <v>207</v>
+        <v>190</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>208</v>
+        <v>191</v>
       </c>
       <c r="B112" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>210</v>
-      </c>
-      <c r="B113" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>212</v>
-      </c>
-      <c r="B114" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>214</v>
-      </c>
-      <c r="B115" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>216</v>
-      </c>
-      <c r="B116" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>218</v>
-      </c>
-      <c r="B117" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>220</v>
-      </c>
-      <c r="B118" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>222</v>
-      </c>
-      <c r="B119" t="s">
         <v>223</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>224</v>
-      </c>
-      <c r="B120" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>226</v>
-      </c>
-      <c r="B121" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>228</v>
-      </c>
-      <c r="B122" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>23</v>
-      </c>
-      <c r="B123" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
-        <v>230</v>
-      </c>
-      <c r="B124" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>232</v>
-      </c>
-      <c r="B125" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
-        <v>234</v>
-      </c>
-      <c r="B126" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
-        <v>236</v>
-      </c>
-      <c r="B127" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
-        <v>280</v>
-      </c>
-      <c r="B128" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
-        <v>238</v>
-      </c>
-      <c r="B129" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
-        <v>240</v>
-      </c>
-      <c r="B130" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
-        <v>242</v>
-      </c>
-      <c r="B131" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
-        <v>244</v>
-      </c>
-      <c r="B132" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
-        <v>246</v>
-      </c>
-      <c r="B133" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
-        <v>284</v>
-      </c>
-      <c r="B134" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
-        <v>248</v>
-      </c>
-      <c r="B135" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
-        <v>250</v>
-      </c>
-      <c r="B136" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
-        <v>288</v>
-      </c>
-      <c r="B137" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
-        <v>286</v>
-      </c>
-      <c r="B138" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
-        <v>290</v>
-      </c>
-      <c r="B139" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
-        <v>292</v>
-      </c>
-      <c r="B140" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A141" t="s">
-        <v>134</v>
-      </c>
-      <c r="B141" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A142" t="s">
-        <v>294</v>
-      </c>
-      <c r="B142" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A143" t="s">
-        <v>296</v>
-      </c>
-      <c r="B143" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A144" t="s">
-        <v>252</v>
-      </c>
-      <c r="B144" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A145" t="s">
-        <v>254</v>
-      </c>
-      <c r="B145" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A146" t="s">
-        <v>257</v>
-      </c>
-      <c r="B146" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A147" t="s">
-        <v>258</v>
-      </c>
-      <c r="B147" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A148" t="s">
-        <v>260</v>
-      </c>
-      <c r="B148" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>262</v>
-      </c>
-      <c r="B149" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A150" t="s">
-        <v>298</v>
-      </c>
-      <c r="B150" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>300</v>
-      </c>
-      <c r="B151" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A152" t="s">
-        <v>302</v>
-      </c>
-      <c r="B152" t="s">
-        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>